<commit_message>
13-12-2025 updated attendence and backend logic
</commit_message>
<xml_diff>
--- a/master/public/sample_template.xlsx
+++ b/master/public/sample_template.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27726"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Downloads\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D5C0488-FCE2-4B9A-9CFB-EE8361B95D86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="19416" windowHeight="10296" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="-105" windowWidth="19410" windowHeight="10290" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="SampleTemplate" sheetId="1" r:id="rId1"/>
@@ -21,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="72">
   <si>
     <t>Userid</t>
   </si>
@@ -71,33 +65,6 @@
     <t>S1</t>
   </si>
   <si>
-    <t>EVA &amp; Back Sheet</t>
-  </si>
-  <si>
-    <t>Cell Assembly</t>
-  </si>
-  <si>
-    <t>EL-1</t>
-  </si>
-  <si>
-    <t>Layup</t>
-  </si>
-  <si>
-    <t>Lamination</t>
-  </si>
-  <si>
-    <t>Framing</t>
-  </si>
-  <si>
-    <t>IV Testing</t>
-  </si>
-  <si>
-    <t>Final EL</t>
-  </si>
-  <si>
-    <t>Packing</t>
-  </si>
-  <si>
     <t>Line</t>
   </si>
   <si>
@@ -105,12 +72,171 @@
   </si>
   <si>
     <t>B</t>
+  </si>
+  <si>
+    <t>Auto glass loading machine</t>
+  </si>
+  <si>
+    <t>EVA cutting &amp; laying machine</t>
+  </si>
+  <si>
+    <t>Stringers</t>
+  </si>
+  <si>
+    <t>Auto soldering bussing machine</t>
+  </si>
+  <si>
+    <t>PSN,RFID &amp; Description Label Fixing and soldering</t>
+  </si>
+  <si>
+    <t>Auto Taping Machine</t>
+  </si>
+  <si>
+    <t>Manual tapping Operation</t>
+  </si>
+  <si>
+    <t>2nd EPE cutting Machine</t>
+  </si>
+  <si>
+    <t>EPE Cut Piece ,EPE Strip fixing and EPE Allignment</t>
+  </si>
+  <si>
+    <t>Double glass loading</t>
+  </si>
+  <si>
+    <t>Ribbon Bending &amp; Teflon piece placement</t>
+  </si>
+  <si>
+    <t>EL-1 &amp; VI tester</t>
+  </si>
+  <si>
+    <t>Module rework after EL-1</t>
+  </si>
+  <si>
+    <t>Edge sealing machine / Layup Allignment</t>
+  </si>
+  <si>
+    <t>Laminator</t>
+  </si>
+  <si>
+    <t>Pin up &amp; Back inspection</t>
+  </si>
+  <si>
+    <t>Edge seal removal</t>
+  </si>
+  <si>
+    <t>Auto Trimming</t>
+  </si>
+  <si>
+    <t>VI-2</t>
+  </si>
+  <si>
+    <t>EL-2</t>
+  </si>
+  <si>
+    <t>Automatic framing &amp; gluing machine</t>
+  </si>
+  <si>
+    <t>After framing inspection &amp; Cleaning</t>
+  </si>
+  <si>
+    <t>JB fixing &amp; JB Sealent despencing</t>
+  </si>
+  <si>
+    <t>JB Soldering &amp; Voltage verification</t>
+  </si>
+  <si>
+    <t>JB Cap fixing</t>
+  </si>
+  <si>
+    <t>Testing tools installation</t>
+  </si>
+  <si>
+    <t>Cleaning</t>
+  </si>
+  <si>
+    <t>Flasher</t>
+  </si>
+  <si>
+    <t>EL-3</t>
+  </si>
+  <si>
+    <t>RFID</t>
+  </si>
+  <si>
+    <t>Testing tools removal &amp; Moving back to loading area</t>
+  </si>
+  <si>
+    <t>VI-3</t>
+  </si>
+  <si>
+    <t>Back Label &amp; Bar code Label printing</t>
+  </si>
+  <si>
+    <t>Corner Cap ,Label Fixing &amp; Back side Barcode Removal</t>
+  </si>
+  <si>
+    <t>Sorting</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SAP posting and FTR preparation </t>
+  </si>
+  <si>
+    <t xml:space="preserve">EL,RFID &amp; IV Curve boxwise updation </t>
+  </si>
+  <si>
+    <t>Packing - sorting Trolley Movemement , Unloading , stacker operation, sleeve fixing &amp; strapping</t>
+  </si>
+  <si>
+    <t>Rfid Mounting</t>
+  </si>
+  <si>
+    <t>Task force team</t>
+  </si>
+  <si>
+    <t>Line Manager</t>
+  </si>
+  <si>
+    <t>Line Engineer</t>
+  </si>
+  <si>
+    <t>Zone leader  - Pre Lamination</t>
+  </si>
+  <si>
+    <t>Spare</t>
+  </si>
+  <si>
+    <t>Zone Leader - Lamination &amp; Framing Line</t>
+  </si>
+  <si>
+    <t>Zone Leader - Testing &amp; Packing Line</t>
+  </si>
+  <si>
+    <t>PSN Mounting</t>
+  </si>
+  <si>
+    <t>Hipot</t>
+  </si>
+  <si>
+    <t>Software Co-ordinators &amp; job card entry</t>
+  </si>
+  <si>
+    <t>Box movement</t>
+  </si>
+  <si>
+    <t>Extra EVA Edge cutting</t>
+  </si>
+  <si>
+    <t>Jig Movement</t>
+  </si>
+  <si>
+    <t>Module Cleaning</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
@@ -120,27 +246,22 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <sz val="10"/>
+      <sz val="11"/>
       <color theme="1"/>
-      <name val="Arial"/>
+      <name val="Calibri"/>
       <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFF0F0F0"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -148,36 +269,24 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right/>
-      <top/>
-      <bottom style="medium">
-        <color rgb="FFDDDDDD"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal 2" xfId="1"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleMedium4"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
-    </ext>
-    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
-      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -504,17 +613,17 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:K2"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="23.19921875" customWidth="1"/>
-    <col min="3" max="3" width="20.59765625" customWidth="1"/>
-    <col min="4" max="4" width="8.69921875" customWidth="1"/>
-    <col min="5" max="11" width="10.09765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="23.25" customWidth="1"/>
+    <col min="3" max="3" width="20.625" customWidth="1"/>
+    <col min="4" max="4" width="8.75" customWidth="1"/>
+    <col min="5" max="11" width="10.125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -525,7 +634,7 @@
         <v>2</v>
       </c>
       <c r="D1" t="s">
-        <v>25</v>
+        <v>16</v>
       </c>
       <c r="E1" t="s">
         <v>3</v>
@@ -549,7 +658,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>74</v>
       </c>
@@ -560,7 +669,7 @@
         <v>11</v>
       </c>
       <c r="D2" t="s">
-        <v>26</v>
+        <v>17</v>
       </c>
       <c r="E2" t="s">
         <v>12</v>
@@ -586,23 +695,24 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
   <ignoredErrors>
     <ignoredError sqref="A1:B2 E1:K2" numberStoredAsText="1"/>
   </ignoredErrors>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
       <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{AEB7599A-4760-4552-96A0-0F684AB86BA1}">
-          <x14:formula1>
-            <xm:f>Sheet1!$B$1:$B$10</xm:f>
-          </x14:formula1>
-          <xm:sqref>C1:C900</xm:sqref>
-        </x14:dataValidation>
-        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{CC420C79-D6F1-422D-8AAC-3ACA08214606}">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
           <x14:formula1>
             <xm:f>Sheet1!$D$1:$D$2</xm:f>
           </x14:formula1>
           <xm:sqref>D1:D1048576</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1">
+          <x14:formula1>
+            <xm:f>Sheet1!$B$1:$B$53</xm:f>
+          </x14:formula1>
+          <xm:sqref>C1:C1048576</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -611,94 +721,442 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{76F5143E-68BF-4C04-81D7-F3716C479C60}">
-  <dimension ref="A1:D10"/>
-  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:D53"/>
+  <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="2.625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="76.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1">
         <v>1</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>56</v>
+      </c>
+      <c r="B2" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>57</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>4</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="1">
+        <v>5</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="1">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="1">
+        <v>7</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="1">
+        <v>8</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>9</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>10</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
         <v>11</v>
       </c>
-      <c r="D1" t="s">
+      <c r="B11" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="1">
+        <v>12</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="1">
+        <v>13</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="1">
+        <v>14</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="1">
+        <v>15</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="1">
+        <v>16</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A17" s="1">
+        <v>17</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A18" s="1">
+        <v>51</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A19" s="1">
+        <v>18</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A20" s="1">
+        <v>19</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A21" s="1">
+        <v>20</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A22" s="1">
+        <v>21</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A23" s="1">
+        <v>22</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A24" s="1">
+        <v>23</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A25" s="1">
+        <v>24</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A26" s="1">
+        <v>25</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A27" s="1">
         <v>26</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="1">
-        <v>2</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D2" t="s">
+      <c r="B27" s="1" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A28" s="1">
         <v>27</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="40.200000000000003" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="1">
-        <v>3</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="1">
-        <v>5</v>
-      </c>
-      <c r="B4" s="1" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="1">
-        <v>6</v>
-      </c>
-      <c r="B5" s="1" t="s">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="6" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A6" s="1">
-        <v>7</v>
-      </c>
-      <c r="B6" s="1" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A7" s="1">
-        <v>8</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>21</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="27" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A8" s="1">
-        <v>9</v>
-      </c>
-      <c r="B8" s="1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A9" s="1">
-        <v>10</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>23</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A10" s="1">
-        <v>11</v>
-      </c>
-      <c r="B10" s="1" t="s">
-        <v>24</v>
+      <c r="B28" s="1" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A29" s="1">
+        <v>28</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A30" s="1">
+        <v>29</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A31" s="1">
+        <v>30</v>
+      </c>
+      <c r="B31" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A32" s="1">
+        <v>31</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A33" s="1">
+        <v>32</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A34" s="1">
+        <v>33</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A35" s="1">
+        <v>34</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A36" s="1">
+        <v>35</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A37" s="1">
+        <v>36</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A38" s="1">
+        <v>37</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A39" s="1">
+        <v>38</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A40" s="1">
+        <v>39</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A41" s="1">
+        <v>40</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A42" s="1">
+        <v>41</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A43" s="1">
+        <v>42</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A44" s="1">
+        <v>43</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A45" s="1">
+        <v>45</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A46" s="1">
+        <v>46</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A47" s="1">
+        <v>47</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A48" s="1">
+        <v>49</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A49" s="1">
+        <v>50</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A50" s="1">
+        <v>52</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A51" s="1">
+        <v>53</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A52" s="1">
+        <v>54</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A53" s="1">
+        <v>65</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>71</v>
       </c>
     </row>
   </sheetData>

</xml_diff>